<commit_message>
docs: add open-access PDF for N26 Bolzenkötter et al. (2025)
PMC 오픈 액세스 데이터(PMC12209136, CC BY 4.0, 출판본)에서 PDF를 받아
00_original_PDF에 추가하고 N26을 확보로 옮깁니다. MD5는 PMC 메타데이터와 일치합니다.

- 마스터 N26 행 확인 상태: Europe PMC 초록 → 원문 PDF 확인, 개입 표현 보강(3분 오디오 안내)
- 미확보 목록에서 N26 제거 → 15편
- 루트 엑셀 '추가 우선 검토 연구' N01의 레포 PDF 파일명 기입
- README 수치 갱신(82편 = 확보 67편 + 미확보 15편)

Refs #7

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/LUMI_RAW데이터 링크.xlsx
+++ b/LUMI_RAW데이터 링크.xlsx
@@ -673,19 +673,19 @@
           <t>LUMI | 36편 근거 적합성 재평가 (기존 34편 + GitHub 저장소 누락 2편)</t>
         </is>
       </c>
-      <c r="B1" s="7" t="n"/>
-      <c r="C1" s="7" t="n"/>
-      <c r="D1" s="7" t="n"/>
-      <c r="E1" s="7" t="n"/>
-      <c r="F1" s="7" t="n"/>
-      <c r="G1" s="7" t="n"/>
-      <c r="H1" s="7" t="n"/>
-      <c r="I1" s="7" t="n"/>
-      <c r="J1" s="7" t="n"/>
-      <c r="K1" s="7" t="n"/>
-      <c r="L1" s="7" t="n"/>
-      <c r="M1" s="7" t="n"/>
-      <c r="N1" s="7" t="n"/>
+      <c r="B1" s="1" t="n"/>
+      <c r="C1" s="1" t="n"/>
+      <c r="D1" s="1" t="n"/>
+      <c r="E1" s="1" t="n"/>
+      <c r="F1" s="1" t="n"/>
+      <c r="G1" s="1" t="n"/>
+      <c r="H1" s="1" t="n"/>
+      <c r="I1" s="1" t="n"/>
+      <c r="J1" s="1" t="n"/>
+      <c r="K1" s="1" t="n"/>
+      <c r="L1" s="1" t="n"/>
+      <c r="M1" s="1" t="n"/>
+      <c r="N1" s="1" t="n"/>
     </row>
     <row r="2" ht="30" customHeight="1" s="40">
       <c r="A2" s="13" t="inlineStr">
@@ -693,19 +693,19 @@
           <t>주의: 직접 근거 여부는 자극 매체·활동 순서·기간·측정 지표의 일치 여부에 따라 판단합니다. 특히 컬러링의 부정 정서 완화 ≠ 반추 감소입니다.</t>
         </is>
       </c>
-      <c r="B2" s="13" t="n"/>
-      <c r="C2" s="13" t="n"/>
-      <c r="D2" s="13" t="n"/>
-      <c r="E2" s="13" t="n"/>
-      <c r="F2" s="13" t="n"/>
-      <c r="G2" s="13" t="n"/>
-      <c r="H2" s="13" t="n"/>
-      <c r="I2" s="13" t="n"/>
-      <c r="J2" s="13" t="n"/>
-      <c r="K2" s="13" t="n"/>
-      <c r="L2" s="13" t="n"/>
-      <c r="M2" s="13" t="n"/>
-      <c r="N2" s="13" t="n"/>
+      <c r="B2" s="1" t="n"/>
+      <c r="C2" s="1" t="n"/>
+      <c r="D2" s="1" t="n"/>
+      <c r="E2" s="1" t="n"/>
+      <c r="F2" s="1" t="n"/>
+      <c r="G2" s="1" t="n"/>
+      <c r="H2" s="1" t="n"/>
+      <c r="I2" s="1" t="n"/>
+      <c r="J2" s="1" t="n"/>
+      <c r="K2" s="1" t="n"/>
+      <c r="L2" s="1" t="n"/>
+      <c r="M2" s="1" t="n"/>
+      <c r="N2" s="1" t="n"/>
     </row>
     <row r="4" ht="28" customHeight="1" s="40">
       <c r="A4" s="16" t="inlineStr">
@@ -3630,14 +3630,14 @@
           <t>LUMI | 사용자 플로우에 직접 가까운 후보 + S1 컬러링/주의 전환 검토 5편</t>
         </is>
       </c>
-      <c r="B1" s="6" t="n"/>
-      <c r="C1" s="6" t="n"/>
-      <c r="D1" s="6" t="n"/>
-      <c r="E1" s="6" t="n"/>
-      <c r="F1" s="6" t="n"/>
-      <c r="G1" s="6" t="n"/>
-      <c r="H1" s="6" t="n"/>
-      <c r="I1" s="6" t="n"/>
+      <c r="B1" s="1" t="n"/>
+      <c r="C1" s="1" t="n"/>
+      <c r="D1" s="1" t="n"/>
+      <c r="E1" s="1" t="n"/>
+      <c r="F1" s="1" t="n"/>
+      <c r="G1" s="1" t="n"/>
+      <c r="H1" s="1" t="n"/>
+      <c r="I1" s="1" t="n"/>
     </row>
     <row r="3" ht="28" customHeight="1" s="40">
       <c r="A3" s="15" t="inlineStr">
@@ -3729,7 +3729,7 @@
       </c>
       <c r="I4" s="21" t="inlineStr">
         <is>
-          <t>미확보</t>
+          <t>N26_2025_Bolzenk_tter_Impact_of_a_Momentary_Mindfulness_Intervention_on_Rumination_Negative.pdf</t>
         </is>
       </c>
     </row>
@@ -4257,7 +4257,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L35"/>
+  <dimension ref="A1:K35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" style="40" min="1" max="1"/>
@@ -6095,7 +6095,6 @@
       <c r="E2" s="1" t="n"/>
       <c r="F2" s="1" t="n"/>
     </row>
-    <row r="3"/>
     <row r="4" ht="26" customHeight="1" s="40">
       <c r="A4" s="61" t="inlineStr">
         <is>
@@ -6218,7 +6217,6 @@
         </is>
       </c>
     </row>
-    <row r="12"/>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
@@ -6249,7 +6247,6 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16"/>
     <row r="17">
       <c r="A17" s="61" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
docs: add P37-P39 publisher PDFs via institutional access
미확보였던 36편 근거 목록 논문 3편을 기관 구독(인천대학교) ScienceDirect
출판본 텍스트 PDF로 추가합니다.

- P37 Laumann et al. (2003), JEP, 10쪽 (36편 목록 P06)
- P38 Lymeus et al. (2018), Consciousness and Cognition, 17쪽 (36편 목록 P12)
- P39 Lymeus et al. (2019), JEP, 9쪽 (36편 목록 P13)

엑셀·README 반영:
- 마스터 해당 행 확인 상태 → 원문 PDF 확인
- 원문 확보 후 채우기로 남긴 칸을 원문 기준으로 기재
  (P37 결과요약·자극 조건, P39 측정 지표·결과요약)
- 루트 엑셀 '34편 근거 재분류' P06·P12·P13의 레포 PDF 파일명 기입
- 미확보 목록에서 3편 제거 → 12편
- README 수치 갱신(82편 = 확보 70편 + 미확보 12편)

Refs #13

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/LUMI_RAW데이터 링크.xlsx
+++ b/LUMI_RAW데이터 링크.xlsx
@@ -1207,7 +1207,7 @@
       </c>
       <c r="N10" s="21" t="inlineStr">
         <is>
-          <t>미확보</t>
+          <t>P37_2003_Laumann_Selective_attention_and_heart_rate_responses_to_natural_and_urban_envi.pdf</t>
         </is>
       </c>
     </row>
@@ -1639,7 +1639,7 @@
       </c>
       <c r="N16" s="21" t="inlineStr">
         <is>
-          <t>미확보</t>
+          <t>P38_2018_Lymeus_Building_mindfulness_bottom_up_Meditation_in_natural_settings_supports.pdf</t>
         </is>
       </c>
     </row>
@@ -1711,7 +1711,7 @@
       </c>
       <c r="N17" s="21" t="inlineStr">
         <is>
-          <t>미확보</t>
+          <t>P39_2019_Lymeus_A_natural_meditation_setting_improves_compliance_with_mindfulness_trai.pdf</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: unify 72 paper-type labels into six study-design categories
- R/C 마스터 엑셀 두 시트에 연구 설계 6범주 `논문 유형` 열 추가, 기존 72종 라벨은 `세부 설계` 열로 보존
- 범주 정의·편수·경계 사례 13건을 담은 `논문 유형 기준` 시트 추가
- 루트 `LUMI_RAW데이터 링크.xlsx`의 `Raw Data 확보 실사` 시트도 같은 6범주 열 추가(36-ID → 마스터 ID 교차표로 매핑)
- README에 열 구조 설명 추가

Closes #19

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/LUMI_RAW데이터 링크.xlsx
+++ b/LUMI_RAW데이터 링크.xlsx
@@ -4257,20 +4257,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K35"/>
+  <dimension ref="A1:L35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" style="40" min="1" max="1"/>
     <col width="22" customWidth="1" style="40" min="2" max="2"/>
     <col width="55" customWidth="1" style="40" min="3" max="3"/>
-    <col width="21" customWidth="1" style="40" min="4" max="4"/>
-    <col width="25" customWidth="1" style="40" min="5" max="5"/>
-    <col width="39" customWidth="1" style="40" min="6" max="6"/>
-    <col width="65" customWidth="1" style="40" min="7" max="7"/>
-    <col width="57" customWidth="1" style="40" min="8" max="8"/>
-    <col width="52" customWidth="1" style="40" min="9" max="9"/>
-    <col width="43" customWidth="1" style="40" min="10" max="10"/>
-    <col width="11" customWidth="1" style="40" min="11" max="11"/>
+    <col width="20" customWidth="1" style="40" min="4" max="4"/>
+    <col width="21" customWidth="1" style="40" min="5" max="5"/>
+    <col width="25" customWidth="1" style="40" min="6" max="6"/>
+    <col width="39" customWidth="1" style="40" min="7" max="7"/>
+    <col width="65" customWidth="1" style="40" min="8" max="8"/>
+    <col width="57" customWidth="1" style="40" min="9" max="9"/>
+    <col width="52" customWidth="1" style="40" min="10" max="10"/>
+    <col width="43" customWidth="1" style="40" min="11" max="11"/>
+    <col width="11" customWidth="1" style="40" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1" s="40">
@@ -4289,6 +4290,7 @@
       <c r="I1" s="1" t="n"/>
       <c r="J1" s="1" t="n"/>
       <c r="K1" s="1" t="n"/>
+      <c r="L1" s="1" t="n"/>
     </row>
     <row r="2" ht="30" customHeight="1" s="40">
       <c r="A2" s="48" t="inlineStr">
@@ -4306,11 +4308,12 @@
       <c r="I2" s="1" t="n"/>
       <c r="J2" s="1" t="n"/>
       <c r="K2" s="1" t="n"/>
+      <c r="L2" s="1" t="n"/>
     </row>
     <row r="3" ht="26" customHeight="1" s="40">
       <c r="A3" s="49" t="inlineStr">
         <is>
-          <t>ID는 '34편 근거 재분류' 시트(36편) 기준으로 바꿨습니다(2026-10-23). 2026-10-21 조사는 당시 목록 31행 대상이며, 같은 리뷰였던 옛 P04·P09는 P35 Ohly et al. (2016) 한 행으로 합쳤습니다. 36편 목록의 P21·P30~P34는 이 조사에 포함되지 않았습니다.</t>
+          <t>ID는 '34편 근거 재분류' 시트(36편) 기준으로 바꿨습니다(2026-10-23). 2026-10-21 조사는 당시 목록 31행 대상이며, 같은 리뷰였던 옛 P04·P09는 P35 Ohly et al. (2016) 한 행으로 합쳤습니다. 36편 목록의 P21·P30~P34는 이 조사에 포함되지 않았습니다. 2026-10-23: '논문 유형' 열(연구 설계 6범주, 기준은 R/C 마스터 엑셀 '논문 유형 기준' 시트)을 추가하고 기존 '연구 유형'은 '세부 설계'로 이름을 바꿨습니다.</t>
         </is>
       </c>
       <c r="B3" s="1" t="n"/>
@@ -4323,6 +4326,7 @@
       <c r="I3" s="1" t="n"/>
       <c r="J3" s="1" t="n"/>
       <c r="K3" s="1" t="n"/>
+      <c r="L3" s="1" t="n"/>
     </row>
     <row r="4" ht="30" customHeight="1" s="40">
       <c r="A4" s="50" t="inlineStr">
@@ -4342,40 +4346,45 @@
       </c>
       <c r="D4" s="50" t="inlineStr">
         <is>
-          <t>연구 유형</t>
+          <t>논문 유형</t>
         </is>
       </c>
       <c r="E4" s="50" t="inlineStr">
         <is>
+          <t>세부 설계</t>
+        </is>
+      </c>
+      <c r="F4" s="50" t="inlineStr">
+        <is>
           <t>참가자별 RAW 상태</t>
         </is>
       </c>
-      <c r="F4" s="50" t="inlineStr">
+      <c r="G4" s="50" t="inlineStr">
         <is>
           <t>확보 가능한 기타 자료</t>
         </is>
       </c>
-      <c r="G4" s="50" t="inlineStr">
+      <c r="H4" s="50" t="inlineStr">
         <is>
           <t>근거 및 주의사항</t>
         </is>
       </c>
-      <c r="H4" s="50" t="inlineStr">
+      <c r="I4" s="50" t="inlineStr">
         <is>
           <t>원자료/보충자료 URL</t>
         </is>
       </c>
-      <c r="I4" s="50" t="inlineStr">
+      <c r="J4" s="50" t="inlineStr">
         <is>
           <t>확인 근거 URL</t>
         </is>
       </c>
-      <c r="J4" s="50" t="inlineStr">
+      <c r="K4" s="50" t="inlineStr">
         <is>
           <t>다음 조치</t>
         </is>
       </c>
-      <c r="K4" s="50" t="inlineStr">
+      <c r="L4" s="50" t="inlineStr">
         <is>
           <t>확인 수준</t>
         </is>
@@ -4399,36 +4408,41 @@
       </c>
       <c r="D5" s="21" t="inlineStr">
         <is>
+          <t>이론·개념 리뷰</t>
+        </is>
+      </c>
+      <c r="E5" s="21" t="inlineStr">
+        <is>
           <t>이론 논문</t>
         </is>
       </c>
-      <c r="E5" s="51" t="inlineStr">
+      <c r="F5" s="51" t="inlineStr">
         <is>
           <t>리뷰/이론 (IPD 비대상)</t>
         </is>
       </c>
-      <c r="F5" s="21" t="inlineStr">
+      <c r="G5" s="21" t="inlineStr">
         <is>
           <t>논문 전문·이론 구조</t>
         </is>
       </c>
-      <c r="G5" s="21" t="inlineStr">
+      <c r="H5" s="21" t="inlineStr">
         <is>
           <t>신규 참가자 실험이 없는 이론적 논문. 독립 IPD 없음</t>
         </is>
       </c>
-      <c r="H5" s="21" t="n"/>
-      <c r="I5" s="21" t="inlineStr">
+      <c r="I5" s="21" t="n"/>
+      <c r="J5" s="21" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/0272-4944(95)90001-2</t>
         </is>
       </c>
-      <c r="J5" s="21" t="inlineStr">
+      <c r="K5" s="21" t="inlineStr">
         <is>
           <t>논문 원문을 ART 근거로 색인</t>
         </is>
       </c>
-      <c r="K5" s="21" t="inlineStr">
+      <c r="L5" s="21" t="inlineStr">
         <is>
           <t>높음</t>
         </is>
@@ -4452,36 +4466,41 @@
       </c>
       <c r="D6" s="52" t="inlineStr">
         <is>
+          <t>무작위 실험</t>
+        </is>
+      </c>
+      <c r="E6" s="52" t="inlineStr">
+        <is>
           <t>시각 실험</t>
         </is>
       </c>
-      <c r="E6" s="53" t="inlineStr">
+      <c r="F6" s="53" t="inlineStr">
         <is>
           <t>참가자 RAW 미확인</t>
         </is>
       </c>
-      <c r="F6" s="52" t="inlineStr">
+      <c r="G6" s="52" t="inlineStr">
         <is>
           <t>본문에 집계·결과</t>
         </is>
       </c>
-      <c r="G6" s="52" t="inlineStr">
+      <c r="H6" s="52" t="inlineStr">
         <is>
           <t>참가자별 주의력 성적 데이터 저장소를 이번 조사에서 확인하지 못함</t>
         </is>
       </c>
-      <c r="H6" s="52" t="n"/>
-      <c r="I6" s="52" t="inlineStr">
+      <c r="I6" s="52" t="n"/>
+      <c r="J6" s="52" t="inlineStr">
         <is>
           <t>https://www.sciencedirect.com/science/article/pii/S0272494405000381</t>
         </is>
       </c>
-      <c r="J6" s="52" t="inlineStr">
+      <c r="K6" s="52" t="inlineStr">
         <is>
           <t>교신저자에게 반응시간·정확도 IPD 요청</t>
         </is>
       </c>
-      <c r="K6" s="52" t="inlineStr">
+      <c r="L6" s="52" t="inlineStr">
         <is>
           <t>중간</t>
         </is>
@@ -4505,36 +4524,41 @@
       </c>
       <c r="D7" s="21" t="inlineStr">
         <is>
+          <t>무작위 실험</t>
+        </is>
+      </c>
+      <c r="E7" s="21" t="inlineStr">
+        <is>
           <t>보행·사진 실험</t>
         </is>
       </c>
-      <c r="E7" s="53" t="inlineStr">
+      <c r="F7" s="53" t="inlineStr">
         <is>
           <t>참가자 RAW 미확인</t>
         </is>
       </c>
-      <c r="F7" s="21" t="inlineStr">
+      <c r="G7" s="21" t="inlineStr">
         <is>
           <t>본문 결과</t>
         </is>
       </c>
-      <c r="G7" s="21" t="inlineStr">
+      <c r="H7" s="21" t="inlineStr">
         <is>
           <t>참가자별 인지과제 결과 데이터 저장소 확인 못함</t>
         </is>
       </c>
-      <c r="H7" s="21" t="n"/>
-      <c r="I7" s="21" t="inlineStr">
+      <c r="I7" s="21" t="n"/>
+      <c r="J7" s="21" t="inlineStr">
         <is>
           <t>https://doi.org/10.1111/j.1467-9280.2008.02225.x</t>
         </is>
       </c>
-      <c r="J7" s="21" t="inlineStr">
+      <c r="K7" s="21" t="inlineStr">
         <is>
           <t>저자에게 두 실험별 데이터 별도 요청</t>
         </is>
       </c>
-      <c r="K7" s="21" t="inlineStr">
+      <c r="L7" s="21" t="inlineStr">
         <is>
           <t>중간</t>
         </is>
@@ -4558,36 +4582,41 @@
       </c>
       <c r="D8" s="52" t="inlineStr">
         <is>
+          <t>체계적 고찰·메타분석</t>
+        </is>
+      </c>
+      <c r="E8" s="52" t="inlineStr">
+        <is>
           <t>메타분석</t>
         </is>
       </c>
-      <c r="E8" s="51" t="inlineStr">
+      <c r="F8" s="51" t="inlineStr">
         <is>
           <t>리뷰/이론 (IPD 비대상)</t>
         </is>
       </c>
-      <c r="F8" s="52" t="inlineStr">
+      <c r="G8" s="52" t="inlineStr">
         <is>
           <t>논문 표·요약통계</t>
         </is>
       </c>
-      <c r="G8" s="52" t="inlineStr">
+      <c r="H8" s="52" t="inlineStr">
         <is>
           <t>참가자별 원자료가 아니라 포함 연구의 추출 효과크기 데이터가 대상. 공개 별도 추출표는 확인 못함</t>
         </is>
       </c>
-      <c r="H8" s="52" t="n"/>
-      <c r="I8" s="52" t="inlineStr">
+      <c r="I8" s="52" t="n"/>
+      <c r="J8" s="52" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/j.jenvp.2025.102632</t>
         </is>
       </c>
-      <c r="J8" s="52" t="inlineStr">
+      <c r="K8" s="52" t="inlineStr">
         <is>
           <t>보충자료에서 추출표 유무 확인</t>
         </is>
       </c>
-      <c r="K8" s="52" t="inlineStr">
+      <c r="L8" s="52" t="inlineStr">
         <is>
           <t>중간</t>
         </is>
@@ -4611,36 +4640,41 @@
       </c>
       <c r="D9" s="21" t="inlineStr">
         <is>
+          <t>무작위 실험</t>
+        </is>
+      </c>
+      <c r="E9" s="21" t="inlineStr">
+        <is>
           <t>현장 보행 실험</t>
         </is>
       </c>
-      <c r="E9" s="53" t="inlineStr">
+      <c r="F9" s="53" t="inlineStr">
         <is>
           <t>참가자 RAW 미확인</t>
         </is>
       </c>
-      <c r="F9" s="21" t="inlineStr">
+      <c r="G9" s="21" t="inlineStr">
         <is>
           <t>집계·생리/주의 결과</t>
         </is>
       </c>
-      <c r="G9" s="21" t="inlineStr">
+      <c r="H9" s="21" t="inlineStr">
         <is>
           <t>112명 실험의 참가자별 혈압·인지 성적 저장소 확인 못함</t>
         </is>
       </c>
-      <c r="H9" s="21" t="n"/>
-      <c r="I9" s="21" t="inlineStr">
+      <c r="I9" s="21" t="n"/>
+      <c r="J9" s="21" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/S0272-4944(02)00109-3</t>
         </is>
       </c>
-      <c r="J9" s="21" t="inlineStr">
+      <c r="K9" s="21" t="inlineStr">
         <is>
           <t>저자 요청 또는 재현 연구 이용</t>
         </is>
       </c>
-      <c r="K9" s="21" t="inlineStr">
+      <c r="L9" s="21" t="inlineStr">
         <is>
           <t>중간</t>
         </is>
@@ -4664,36 +4698,41 @@
       </c>
       <c r="D10" s="52" t="inlineStr">
         <is>
+          <t>무작위 실험</t>
+        </is>
+      </c>
+      <c r="E10" s="52" t="inlineStr">
+        <is>
           <t>영상 실험</t>
         </is>
       </c>
-      <c r="E10" s="53" t="inlineStr">
+      <c r="F10" s="53" t="inlineStr">
         <is>
           <t>참가자 RAW 미확인</t>
         </is>
       </c>
-      <c r="F10" s="52" t="inlineStr">
+      <c r="G10" s="52" t="inlineStr">
         <is>
           <t>본문 결과</t>
         </is>
       </c>
-      <c r="G10" s="52" t="inlineStr">
+      <c r="H10" s="52" t="inlineStr">
         <is>
           <t>선택주의·심박 원자료 저장소 확인 못함</t>
         </is>
       </c>
-      <c r="H10" s="52" t="n"/>
-      <c r="I10" s="52" t="inlineStr">
+      <c r="I10" s="52" t="n"/>
+      <c r="J10" s="52" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/S0272-4944(02)00110-X</t>
         </is>
       </c>
-      <c r="J10" s="52" t="inlineStr">
+      <c r="K10" s="52" t="inlineStr">
         <is>
           <t>저자에게 IPD 및 자극 영상 문의</t>
         </is>
       </c>
-      <c r="K10" s="52" t="inlineStr">
+      <c r="L10" s="52" t="inlineStr">
         <is>
           <t>중간</t>
         </is>
@@ -4717,36 +4756,41 @@
       </c>
       <c r="D11" s="21" t="inlineStr">
         <is>
+          <t>무작위 실험</t>
+        </is>
+      </c>
+      <c r="E11" s="21" t="inlineStr">
+        <is>
           <t>시청각 스트레스 실험</t>
         </is>
       </c>
-      <c r="E11" s="53" t="inlineStr">
+      <c r="F11" s="53" t="inlineStr">
         <is>
           <t>참가자 RAW 미확인</t>
         </is>
       </c>
-      <c r="F11" s="21" t="inlineStr">
+      <c r="G11" s="21" t="inlineStr">
         <is>
           <t>논문 및 집계 결과</t>
         </is>
       </c>
-      <c r="G11" s="21" t="inlineStr">
+      <c r="H11" s="21" t="inlineStr">
         <is>
           <t>원전 참가자별 스트레스·생리 신호 자료 공개 링크 확인 못함</t>
         </is>
       </c>
-      <c r="H11" s="21" t="n"/>
-      <c r="I11" s="21" t="inlineStr">
+      <c r="I11" s="21" t="n"/>
+      <c r="J11" s="21" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/S0272-4944(05)80184-7</t>
         </is>
       </c>
-      <c r="J11" s="21" t="inlineStr">
+      <c r="K11" s="21" t="inlineStr">
         <is>
           <t>원전 저자 또는 2026 재현연구 검토</t>
         </is>
       </c>
-      <c r="K11" s="21" t="inlineStr">
+      <c r="L11" s="21" t="inlineStr">
         <is>
           <t>중간</t>
         </is>
@@ -4770,36 +4814,41 @@
       </c>
       <c r="D12" s="52" t="inlineStr">
         <is>
+          <t>무작위 실험</t>
+        </is>
+      </c>
+      <c r="E12" s="52" t="inlineStr">
+        <is>
           <t>자연 이미지·HRV 실험</t>
         </is>
       </c>
-      <c r="E12" s="53" t="inlineStr">
+      <c r="F12" s="53" t="inlineStr">
         <is>
           <t>참가자 RAW 미확인</t>
         </is>
       </c>
-      <c r="F12" s="52" t="inlineStr">
+      <c r="G12" s="52" t="inlineStr">
         <is>
           <t>논문 통계</t>
         </is>
       </c>
-      <c r="G12" s="52" t="inlineStr">
+      <c r="H12" s="52" t="inlineStr">
         <is>
           <t>개인별 HRV/RMSSD 시계열 저장소 확인 못함</t>
         </is>
       </c>
-      <c r="H12" s="52" t="n"/>
-      <c r="I12" s="52" t="inlineStr">
+      <c r="I12" s="52" t="n"/>
+      <c r="J12" s="52" t="inlineStr">
         <is>
           <t>https://doi.org/10.1021/es305019p</t>
         </is>
       </c>
-      <c r="J12" s="52" t="inlineStr">
+      <c r="K12" s="52" t="inlineStr">
         <is>
           <t>교신저자 IPD 요청</t>
         </is>
       </c>
-      <c r="K12" s="52" t="inlineStr">
+      <c r="L12" s="52" t="inlineStr">
         <is>
           <t>중간</t>
         </is>
@@ -4823,40 +4872,45 @@
       </c>
       <c r="D13" s="21" t="inlineStr">
         <is>
+          <t>무작위 실험</t>
+        </is>
+      </c>
+      <c r="E13" s="21" t="inlineStr">
+        <is>
           <t>자연 이미지·fMRI 실험</t>
         </is>
       </c>
-      <c r="E13" s="54" t="inlineStr">
+      <c r="F13" s="54" t="inlineStr">
         <is>
           <t>저자 요청 RAW</t>
         </is>
       </c>
-      <c r="F13" s="21" t="inlineStr">
+      <c r="G13" s="21" t="inlineStr">
         <is>
           <t>보충 Word 자료</t>
         </is>
       </c>
-      <c r="G13" s="21" t="inlineStr">
+      <c r="H13" s="21" t="inlineStr">
         <is>
           <t>논문 Data availability: Data will be made available on request. 공개 RAW 다운로드는 아님</t>
         </is>
       </c>
-      <c r="H13" s="21" t="inlineStr">
+      <c r="I13" s="21" t="inlineStr">
         <is>
           <t>https://www.sciencedirect.com/science/article/pii/S2352289525000530</t>
         </is>
       </c>
-      <c r="I13" s="21" t="inlineStr">
+      <c r="J13" s="21" t="inlineStr">
         <is>
           <t>https://www.sciencedirect.com/science/article/pii/S2352289525000530</t>
         </is>
       </c>
-      <c r="J13" s="21" t="inlineStr">
+      <c r="K13" s="21" t="inlineStr">
         <is>
           <t>교신저자에게 fMRI·정서·코르티솔 비식별 데이터 요청</t>
         </is>
       </c>
-      <c r="K13" s="21" t="inlineStr">
+      <c r="L13" s="21" t="inlineStr">
         <is>
           <t>높음</t>
         </is>
@@ -4880,40 +4934,45 @@
       </c>
       <c r="D14" s="52" t="inlineStr">
         <is>
+          <t>무작위 실험</t>
+        </is>
+      </c>
+      <c r="E14" s="52" t="inlineStr">
+        <is>
           <t>다기관 재현 실험</t>
         </is>
       </c>
-      <c r="E14" s="53" t="inlineStr">
+      <c r="F14" s="53" t="inlineStr">
         <is>
           <t>참가자 RAW 미확인</t>
         </is>
       </c>
-      <c r="F14" s="52" t="inlineStr">
+      <c r="G14" s="52" t="inlineStr">
         <is>
           <t>공개 논문·OSF 사전등록</t>
         </is>
       </c>
-      <c r="G14" s="52" t="inlineStr">
+      <c r="H14" s="52" t="inlineStr">
         <is>
           <t>OSF 사전등록/분석계획 확인. 959명 참가자별 생리·자기보고 RAW 공개 파일은 이번 조사에서 검증 못함</t>
         </is>
       </c>
-      <c r="H14" s="52" t="inlineStr">
+      <c r="I14" s="52" t="inlineStr">
         <is>
           <t>https://osf.io/zhpfd</t>
         </is>
       </c>
-      <c r="I14" s="52" t="inlineStr">
+      <c r="J14" s="52" t="inlineStr">
         <is>
           <t>https://www.sciencedirect.com/science/article/pii/S0272494426000575</t>
         </is>
       </c>
-      <c r="J14" s="52" t="inlineStr">
+      <c r="K14" s="52" t="inlineStr">
         <is>
           <t>OSF files/Data availability 세부 확인; 연구진 문의</t>
         </is>
       </c>
-      <c r="K14" s="52" t="inlineStr">
+      <c r="L14" s="52" t="inlineStr">
         <is>
           <t>중간</t>
         </is>
@@ -4937,36 +4996,41 @@
       </c>
       <c r="D15" s="21" t="inlineStr">
         <is>
+          <t>관찰·설문·질적 연구</t>
+        </is>
+      </c>
+      <c r="E15" s="21" t="inlineStr">
+        <is>
           <t>수술 환자 관찰 연구</t>
         </is>
       </c>
-      <c r="E15" s="53" t="inlineStr">
+      <c r="F15" s="53" t="inlineStr">
         <is>
           <t>참가자 RAW 미확인</t>
         </is>
       </c>
-      <c r="F15" s="21" t="inlineStr">
+      <c r="G15" s="21" t="inlineStr">
         <is>
           <t>논문 결과</t>
         </is>
       </c>
-      <c r="G15" s="21" t="inlineStr">
+      <c r="H15" s="21" t="inlineStr">
         <is>
           <t>1984년 연구의 환자별 기록 데이터 공개 저장소 확인 못함</t>
         </is>
       </c>
-      <c r="H15" s="21" t="n"/>
-      <c r="I15" s="21" t="inlineStr">
+      <c r="I15" s="21" t="n"/>
+      <c r="J15" s="21" t="inlineStr">
         <is>
           <t>https://doi.org/10.1126/science.6143402</t>
         </is>
       </c>
-      <c r="J15" s="21" t="inlineStr">
+      <c r="K15" s="21" t="inlineStr">
         <is>
           <t>원본 자료 활용 대신 집계 결과만 인덱싱</t>
         </is>
       </c>
-      <c r="K15" s="21" t="inlineStr">
+      <c r="L15" s="21" t="inlineStr">
         <is>
           <t>중간</t>
         </is>
@@ -4990,40 +5054,45 @@
       </c>
       <c r="D16" s="52" t="inlineStr">
         <is>
+          <t>무작위 실험</t>
+        </is>
+      </c>
+      <c r="E16" s="52" t="inlineStr">
+        <is>
           <t>ReST 인지과제 실험</t>
         </is>
       </c>
-      <c r="E16" s="53" t="inlineStr">
+      <c r="F16" s="53" t="inlineStr">
         <is>
           <t>참가자 RAW 미확인</t>
         </is>
       </c>
-      <c r="F16" s="52" t="inlineStr">
+      <c r="G16" s="52" t="inlineStr">
         <is>
           <t>논문 결과</t>
         </is>
       </c>
-      <c r="G16" s="52" t="inlineStr">
+      <c r="H16" s="52" t="inlineStr">
         <is>
           <t>같은 연구 프로그램 ReST 2020 데이터셋 존재하지만 P15의 개별 인지과제 자료 포함 여부는 미확인</t>
         </is>
       </c>
-      <c r="H16" s="52" t="inlineStr">
+      <c r="I16" s="52" t="inlineStr">
         <is>
           <t>https://researchdata.se/en/catalogue/dataset/2020-17-1</t>
         </is>
       </c>
-      <c r="I16" s="52" t="inlineStr">
+      <c r="J16" s="52" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/j.concog.2018.01.008</t>
         </is>
       </c>
-      <c r="J16" s="52" t="inlineStr">
+      <c r="K16" s="52" t="inlineStr">
         <is>
           <t>Lymeus 연구진에 P12 자료와 SND 데이터셋의 연결 확인</t>
         </is>
       </c>
-      <c r="K16" s="52" t="inlineStr">
+      <c r="L16" s="52" t="inlineStr">
         <is>
           <t>중간</t>
         </is>
@@ -5047,40 +5116,45 @@
       </c>
       <c r="D17" s="21" t="inlineStr">
         <is>
+          <t>무작위 실험</t>
+        </is>
+      </c>
+      <c r="E17" s="21" t="inlineStr">
+        <is>
           <t>ReST 순응도 실험</t>
         </is>
       </c>
-      <c r="E17" s="53" t="inlineStr">
+      <c r="F17" s="53" t="inlineStr">
         <is>
           <t>참가자 RAW 미확인</t>
         </is>
       </c>
-      <c r="F17" s="21" t="inlineStr">
+      <c r="G17" s="21" t="inlineStr">
         <is>
           <t>논문 결과</t>
         </is>
       </c>
-      <c r="G17" s="21" t="inlineStr">
+      <c r="H17" s="21" t="inlineStr">
         <is>
           <t>같은 ReST 연구군 데이터셋 존재하나 P16의 과제 수행·탈락·순응도 원자료 포함 여부 확인 안 됨</t>
         </is>
       </c>
-      <c r="H17" s="21" t="inlineStr">
+      <c r="I17" s="21" t="inlineStr">
         <is>
           <t>https://researchdata.se/en/catalogue/dataset/2020-17-1</t>
         </is>
       </c>
-      <c r="I17" s="21" t="inlineStr">
+      <c r="J17" s="21" t="inlineStr">
         <is>
           <t>https://www.sciencedirect.com/science/article/abs/pii/S0272494419300258</t>
         </is>
       </c>
-      <c r="J17" s="21" t="inlineStr">
+      <c r="K17" s="21" t="inlineStr">
         <is>
           <t>데이터 사전 확인 후 ReST 연구진 요청</t>
         </is>
       </c>
-      <c r="K17" s="21" t="inlineStr">
+      <c r="L17" s="21" t="inlineStr">
         <is>
           <t>중간</t>
         </is>
@@ -5104,40 +5178,45 @@
       </c>
       <c r="D18" s="52" t="inlineStr">
         <is>
+          <t>무작위 실험</t>
+        </is>
+      </c>
+      <c r="E18" s="52" t="inlineStr">
+        <is>
           <t>ReST 5주 훈련 실험</t>
         </is>
       </c>
-      <c r="E18" s="55" t="inlineStr">
+      <c r="F18" s="55" t="inlineStr">
         <is>
           <t>제한 접근 RAW</t>
         </is>
       </c>
-      <c r="F18" s="52" t="inlineStr">
+      <c r="G18" s="52" t="inlineStr">
         <is>
           <t>코드북·설명 문서 다운로드 가능</t>
         </is>
       </c>
-      <c r="G18" s="52" t="inlineStr">
+      <c r="H18" s="52" t="inlineStr">
         <is>
           <t>Swedish National Data Service에 개인별 스트레스·인지실수·마음챙김 설문. 건강정보 포함, 접근 제한</t>
         </is>
       </c>
-      <c r="H18" s="52" t="inlineStr">
+      <c r="I18" s="52" t="inlineStr">
         <is>
           <t>https://researchdata.se/en/catalogue/dataset/2020-17-1</t>
         </is>
       </c>
-      <c r="I18" s="52" t="inlineStr">
+      <c r="J18" s="52" t="inlineStr">
         <is>
           <t>https://researchdata.se/en/catalogue/dataset/2020-17-1</t>
         </is>
       </c>
-      <c r="J18" s="52" t="inlineStr">
+      <c r="K18" s="52" t="inlineStr">
         <is>
           <t>이용 목적·보안계획과 함께 접근 신청</t>
         </is>
       </c>
-      <c r="K18" s="52" t="inlineStr">
+      <c r="L18" s="52" t="inlineStr">
         <is>
           <t>높음</t>
         </is>
@@ -5161,40 +5240,45 @@
       </c>
       <c r="D19" s="21" t="inlineStr">
         <is>
+          <t>무작위 실험</t>
+        </is>
+      </c>
+      <c r="E19" s="21" t="inlineStr">
+        <is>
           <t>ReST 6개월 종단추적</t>
         </is>
       </c>
-      <c r="E19" s="55" t="inlineStr">
+      <c r="F19" s="55" t="inlineStr">
         <is>
           <t>제한 접근 RAW</t>
         </is>
       </c>
-      <c r="F19" s="21" t="inlineStr">
+      <c r="G19" s="21" t="inlineStr">
         <is>
           <t>코드북·설명 문서 다운로드 가능</t>
         </is>
       </c>
-      <c r="G19" s="21" t="inlineStr">
+      <c r="H19" s="21" t="inlineStr">
         <is>
           <t>SND 보관: 추적 원자료·다중 대치 데이터. P17과 일부 참가자/변수 중복</t>
         </is>
       </c>
-      <c r="H19" s="21" t="inlineStr">
+      <c r="I19" s="21" t="inlineStr">
         <is>
           <t>https://researchdata.se/en/catalogue/dataset/2020-17-2</t>
         </is>
       </c>
-      <c r="I19" s="21" t="inlineStr">
+      <c r="J19" s="21" t="inlineStr">
         <is>
           <t>https://researchdata.se/en/catalogue/dataset/2020-17-2</t>
         </is>
       </c>
-      <c r="J19" s="21" t="inlineStr">
+      <c r="K19" s="21" t="inlineStr">
         <is>
           <t>접근 신청; P17과 환자·변수 중복 관리</t>
         </is>
       </c>
-      <c r="K19" s="21" t="inlineStr">
+      <c r="L19" s="21" t="inlineStr">
         <is>
           <t>높음</t>
         </is>
@@ -5218,36 +5302,41 @@
       </c>
       <c r="D20" s="52" t="inlineStr">
         <is>
+          <t>체계적 고찰·메타분석</t>
+        </is>
+      </c>
+      <c r="E20" s="52" t="inlineStr">
+        <is>
           <t>메타분석</t>
         </is>
       </c>
-      <c r="E20" s="51" t="inlineStr">
+      <c r="F20" s="51" t="inlineStr">
         <is>
           <t>리뷰/이론 (IPD 비대상)</t>
         </is>
       </c>
-      <c r="F20" s="52" t="inlineStr">
+      <c r="G20" s="52" t="inlineStr">
         <is>
           <t>논문 본문 효과크기·집계</t>
         </is>
       </c>
-      <c r="G20" s="52" t="inlineStr">
+      <c r="H20" s="52" t="inlineStr">
         <is>
           <t>참가자별 IPD가 아닌 포함 연구 추출표. 추출 프로토콜은 교신저자 요청 가능</t>
         </is>
       </c>
-      <c r="H20" s="52" t="n"/>
-      <c r="I20" s="52" t="inlineStr">
+      <c r="I20" s="52" t="n"/>
+      <c r="J20" s="52" t="inlineStr">
         <is>
           <t>https://pmc.ncbi.nlm.nih.gov/articles/PMC6747393/</t>
         </is>
       </c>
-      <c r="J20" s="52" t="inlineStr">
+      <c r="K20" s="52" t="inlineStr">
         <is>
           <t>논문 표 사용; 상세 추출표 저자 요청</t>
         </is>
       </c>
-      <c r="K20" s="52" t="inlineStr">
+      <c r="L20" s="52" t="inlineStr">
         <is>
           <t>높음</t>
         </is>
@@ -5271,40 +5360,45 @@
       </c>
       <c r="D21" s="21" t="inlineStr">
         <is>
+          <t>체계적 고찰·메타분석</t>
+        </is>
+      </c>
+      <c r="E21" s="21" t="inlineStr">
+        <is>
           <t>스코핑 리뷰</t>
         </is>
       </c>
-      <c r="E21" s="51" t="inlineStr">
+      <c r="F21" s="51" t="inlineStr">
         <is>
           <t>리뷰/이론 (IPD 비대상)</t>
         </is>
       </c>
-      <c r="F21" s="21" t="inlineStr">
+      <c r="G21" s="21" t="inlineStr">
         <is>
           <t>공개 보충 DOCX·논문 내 자료</t>
         </is>
       </c>
-      <c r="G21" s="21" t="inlineStr">
+      <c r="H21" s="21" t="inlineStr">
         <is>
           <t>논문 Data Availability: Data available within the article. 참가자별 신규 IPD 없음</t>
         </is>
       </c>
-      <c r="H21" s="21" t="inlineStr">
+      <c r="I21" s="21" t="inlineStr">
         <is>
           <t>https://link.springer.com/article/10.1007/s12671-024-02393-8</t>
         </is>
       </c>
-      <c r="I21" s="21" t="inlineStr">
+      <c r="J21" s="21" t="inlineStr">
         <is>
           <t>https://link.springer.com/article/10.1007/s12671-024-02393-8</t>
         </is>
       </c>
-      <c r="J21" s="21" t="inlineStr">
+      <c r="K21" s="21" t="inlineStr">
         <is>
           <t>보충자료에서 중재 환경 구조 추출</t>
         </is>
       </c>
-      <c r="K21" s="21" t="inlineStr">
+      <c r="L21" s="21" t="inlineStr">
         <is>
           <t>높음</t>
         </is>
@@ -5328,40 +5422,45 @@
       </c>
       <c r="D22" s="52" t="inlineStr">
         <is>
+          <t>체계적 고찰·메타분석</t>
+        </is>
+      </c>
+      <c r="E22" s="52" t="inlineStr">
+        <is>
           <t>메타분석</t>
         </is>
       </c>
-      <c r="E22" s="51" t="inlineStr">
+      <c r="F22" s="51" t="inlineStr">
         <is>
           <t>리뷰/이론 (IPD 비대상)</t>
         </is>
       </c>
-      <c r="F22" s="52" t="inlineStr">
+      <c r="G22" s="52" t="inlineStr">
         <is>
           <t>공개 추출 데이터·보충파일</t>
         </is>
       </c>
-      <c r="G22" s="52" t="inlineStr">
+      <c r="H22" s="52" t="inlineStr">
         <is>
           <t>논문 Data availability에 메타분석 추출 dataset이 supplementary files에 있다고 명시 (참가자 IPD 아님)</t>
         </is>
       </c>
-      <c r="H22" s="52" t="inlineStr">
+      <c r="I22" s="52" t="inlineStr">
         <is>
           <t>https://pmc.ncbi.nlm.nih.gov/articles/PMC12382274/</t>
         </is>
       </c>
-      <c r="I22" s="52" t="inlineStr">
+      <c r="J22" s="52" t="inlineStr">
         <is>
           <t>https://pmc.ncbi.nlm.nih.gov/articles/PMC12382274/</t>
         </is>
       </c>
-      <c r="J22" s="52" t="inlineStr">
+      <c r="K22" s="52" t="inlineStr">
         <is>
           <t>보충 파일 받아 연구별 effect 데이터 추출</t>
         </is>
       </c>
-      <c r="K22" s="52" t="inlineStr">
+      <c r="L22" s="52" t="inlineStr">
         <is>
           <t>높음</t>
         </is>
@@ -5385,40 +5484,45 @@
       </c>
       <c r="D23" s="21" t="inlineStr">
         <is>
+          <t>체계적 고찰·메타분석</t>
+        </is>
+      </c>
+      <c r="E23" s="21" t="inlineStr">
+        <is>
           <t>메타분석</t>
         </is>
       </c>
-      <c r="E23" s="51" t="inlineStr">
+      <c r="F23" s="51" t="inlineStr">
         <is>
           <t>리뷰/이론 (IPD 비대상)</t>
         </is>
       </c>
-      <c r="F23" s="21" t="inlineStr">
+      <c r="G23" s="21" t="inlineStr">
         <is>
           <t>연구별 추출 스프레드시트(저자 공개 명시)</t>
         </is>
       </c>
-      <c r="G23" s="21" t="inlineStr">
+      <c r="H23" s="21" t="inlineStr">
         <is>
           <t>논문이 OSF에 추출 스프레드시트 제공을 명시. 55개 연구의 집계/코딩, 참가자 IPD 아님</t>
         </is>
       </c>
-      <c r="H23" s="21" t="inlineStr">
+      <c r="I23" s="21" t="inlineStr">
         <is>
           <t>https://osf.io/wdbfj</t>
         </is>
       </c>
-      <c r="I23" s="21" t="inlineStr">
+      <c r="J23" s="21" t="inlineStr">
         <is>
           <t>https://pmc.ncbi.nlm.nih.gov/articles/PMC12017360/</t>
         </is>
       </c>
-      <c r="J23" s="21" t="inlineStr">
+      <c r="K23" s="21" t="inlineStr">
         <is>
           <t>OSF 파일 열람 및 CSV/XLSX 확보</t>
         </is>
       </c>
-      <c r="K23" s="21" t="inlineStr">
+      <c r="L23" s="21" t="inlineStr">
         <is>
           <t>높음</t>
         </is>
@@ -5442,40 +5546,45 @@
       </c>
       <c r="D24" s="52" t="inlineStr">
         <is>
+          <t>체계적 고찰·메타분석</t>
+        </is>
+      </c>
+      <c r="E24" s="52" t="inlineStr">
+        <is>
           <t>체계적 문헌고찰</t>
         </is>
       </c>
-      <c r="E24" s="51" t="inlineStr">
+      <c r="F24" s="51" t="inlineStr">
         <is>
           <t>리뷰/이론 (IPD 비대상)</t>
         </is>
       </c>
-      <c r="F24" s="52" t="inlineStr">
+      <c r="G24" s="52" t="inlineStr">
         <is>
           <t>논문 집계·보충 PDF</t>
         </is>
       </c>
-      <c r="G24" s="52" t="inlineStr">
+      <c r="H24" s="52" t="inlineStr">
         <is>
           <t>추가 추출 outcome/앱 참여 지표는 교신저자 요청. 참가자 IPD 아님</t>
         </is>
       </c>
-      <c r="H24" s="52" t="inlineStr">
+      <c r="I24" s="52" t="inlineStr">
         <is>
           <t>https://pmc.ncbi.nlm.nih.gov/articles/PMC10955957/</t>
         </is>
       </c>
-      <c r="I24" s="52" t="inlineStr">
+      <c r="J24" s="52" t="inlineStr">
         <is>
           <t>https://pmc.ncbi.nlm.nih.gov/articles/PMC10955957/</t>
         </is>
       </c>
-      <c r="J24" s="52" t="inlineStr">
+      <c r="K24" s="52" t="inlineStr">
         <is>
           <t>보충표 다운로드·추가 추출표 저자 요청</t>
         </is>
       </c>
-      <c r="K24" s="52" t="inlineStr">
+      <c r="L24" s="52" t="inlineStr">
         <is>
           <t>높음</t>
         </is>
@@ -5499,36 +5608,41 @@
       </c>
       <c r="D25" s="21" t="inlineStr">
         <is>
+          <t>체계적 고찰·메타분석</t>
+        </is>
+      </c>
+      <c r="E25" s="21" t="inlineStr">
+        <is>
           <t>체계적 문헌고찰</t>
         </is>
       </c>
-      <c r="E25" s="51" t="inlineStr">
+      <c r="F25" s="51" t="inlineStr">
         <is>
           <t>리뷰/이론 (IPD 비대상)</t>
         </is>
       </c>
-      <c r="F25" s="21" t="inlineStr">
+      <c r="G25" s="21" t="inlineStr">
         <is>
           <t>공개 논문 집계 결과</t>
         </is>
       </c>
-      <c r="G25" s="21" t="inlineStr">
+      <c r="H25" s="21" t="inlineStr">
         <is>
           <t>리뷰 자체 신규 참가자 RAW 없음. 별도 추출표 공개 여부 확인 못함</t>
         </is>
       </c>
-      <c r="H25" s="21" t="n"/>
-      <c r="I25" s="21" t="inlineStr">
+      <c r="I25" s="21" t="n"/>
+      <c r="J25" s="21" t="inlineStr">
         <is>
           <t>https://doi.org/10.2147/PRBM.S437277</t>
         </is>
       </c>
-      <c r="J25" s="21" t="inlineStr">
+      <c r="K25" s="21" t="inlineStr">
         <is>
           <t>연구별 데이터 추출표 요청</t>
         </is>
       </c>
-      <c r="K25" s="21" t="inlineStr">
+      <c r="L25" s="21" t="inlineStr">
         <is>
           <t>중간</t>
         </is>
@@ -5552,40 +5666,45 @@
       </c>
       <c r="D26" s="52" t="inlineStr">
         <is>
+          <t>체계적 고찰·메타분석</t>
+        </is>
+      </c>
+      <c r="E26" s="52" t="inlineStr">
+        <is>
           <t>메타분석</t>
         </is>
       </c>
-      <c r="E26" s="51" t="inlineStr">
+      <c r="F26" s="51" t="inlineStr">
         <is>
           <t>리뷰/이론 (IPD 비대상)</t>
         </is>
       </c>
-      <c r="F26" s="52" t="inlineStr">
+      <c r="G26" s="52" t="inlineStr">
         <is>
           <t>보충 PDF</t>
         </is>
       </c>
-      <c r="G26" s="52" t="inlineStr">
+      <c r="H26" s="52" t="inlineStr">
         <is>
           <t>논문 Data availability: datasets available from corresponding author on reasonable request. IPD가 아닌 메타분석 데이터</t>
         </is>
       </c>
-      <c r="H26" s="52" t="inlineStr">
+      <c r="I26" s="52" t="inlineStr">
         <is>
           <t>https://pmc.ncbi.nlm.nih.gov/articles/PMC9828383/</t>
         </is>
       </c>
-      <c r="I26" s="52" t="inlineStr">
+      <c r="J26" s="52" t="inlineStr">
         <is>
           <t>https://pmc.ncbi.nlm.nih.gov/articles/PMC9828383/</t>
         </is>
       </c>
-      <c r="J26" s="52" t="inlineStr">
+      <c r="K26" s="52" t="inlineStr">
         <is>
           <t>교신저자에게 메타분석 추출 데이터 요청</t>
         </is>
       </c>
-      <c r="K26" s="52" t="inlineStr">
+      <c r="L26" s="52" t="inlineStr">
         <is>
           <t>높음</t>
         </is>
@@ -5609,40 +5728,45 @@
       </c>
       <c r="D27" s="21" t="inlineStr">
         <is>
+          <t>체계적 고찰·메타분석</t>
+        </is>
+      </c>
+      <c r="E27" s="21" t="inlineStr">
+        <is>
           <t>체계적 문헌고찰</t>
         </is>
       </c>
-      <c r="E27" s="51" t="inlineStr">
+      <c r="F27" s="51" t="inlineStr">
         <is>
           <t>리뷰/이론 (IPD 비대상)</t>
         </is>
       </c>
-      <c r="F27" s="21" t="inlineStr">
+      <c r="G27" s="21" t="inlineStr">
         <is>
           <t>공개 보충 ZIP: 합성 자료·R markdown 출력</t>
         </is>
       </c>
-      <c r="G27" s="21" t="inlineStr">
+      <c r="H27" s="21" t="inlineStr">
         <is>
           <t>Data synthesis/output 보충자료 공개. 기타 자료는 요청. 참가자 IPD 아님</t>
         </is>
       </c>
-      <c r="H27" s="21" t="inlineStr">
+      <c r="I27" s="21" t="inlineStr">
         <is>
           <t>https://pmc.ncbi.nlm.nih.gov/articles/PMC10741869/</t>
         </is>
       </c>
-      <c r="I27" s="21" t="inlineStr">
+      <c r="J27" s="21" t="inlineStr">
         <is>
           <t>https://pmc.ncbi.nlm.nih.gov/articles/PMC10741869/</t>
         </is>
       </c>
-      <c r="J27" s="21" t="inlineStr">
+      <c r="K27" s="21" t="inlineStr">
         <is>
           <t>보충 ZIP 추출해 연구 조건 분류</t>
         </is>
       </c>
-      <c r="K27" s="21" t="inlineStr">
+      <c r="L27" s="21" t="inlineStr">
         <is>
           <t>높음</t>
         </is>
@@ -5666,40 +5790,45 @@
       </c>
       <c r="D28" s="52" t="inlineStr">
         <is>
+          <t>무작위 실험</t>
+        </is>
+      </c>
+      <c r="E28" s="52" t="inlineStr">
+        <is>
           <t>PMR·호흡·유도 심상 실험</t>
         </is>
       </c>
-      <c r="E28" s="54" t="inlineStr">
+      <c r="F28" s="54" t="inlineStr">
         <is>
           <t>저자 요청 RAW</t>
         </is>
       </c>
-      <c r="F28" s="52" t="inlineStr">
+      <c r="G28" s="52" t="inlineStr">
         <is>
           <t>논문 집계·결과</t>
         </is>
       </c>
-      <c r="G28" s="52" t="inlineStr">
+      <c r="H28" s="52" t="inlineStr">
         <is>
           <t>Data Availability: Data are available upon request to the first author</t>
         </is>
       </c>
-      <c r="H28" s="52" t="inlineStr">
+      <c r="I28" s="52" t="inlineStr">
         <is>
           <t>https://pmc.ncbi.nlm.nih.gov/articles/PMC8272667/</t>
         </is>
       </c>
-      <c r="I28" s="52" t="inlineStr">
+      <c r="J28" s="52" t="inlineStr">
         <is>
           <t>https://pmc.ncbi.nlm.nih.gov/articles/PMC8272667/</t>
         </is>
       </c>
-      <c r="J28" s="52" t="inlineStr">
+      <c r="K28" s="52" t="inlineStr">
         <is>
           <t>제1저자에게 익명 설문·심박·피부전도 RAW 요청</t>
         </is>
       </c>
-      <c r="K28" s="52" t="inlineStr">
+      <c r="L28" s="52" t="inlineStr">
         <is>
           <t>높음</t>
         </is>
@@ -5723,40 +5852,45 @@
       </c>
       <c r="D29" s="21" t="inlineStr">
         <is>
+          <t>무작위 실험</t>
+        </is>
+      </c>
+      <c r="E29" s="21" t="inlineStr">
+        <is>
           <t>1개월 호흡 중재 RCT</t>
         </is>
       </c>
-      <c r="E29" s="56" t="inlineStr">
+      <c r="F29" s="56" t="inlineStr">
         <is>
           <t>공개 RAW</t>
         </is>
       </c>
-      <c r="F29" s="21" t="inlineStr">
+      <c r="G29" s="21" t="inlineStr">
         <is>
           <t>분석 R 코드(Zenodo)·논문 보충 PDF</t>
         </is>
       </c>
-      <c r="G29" s="21" t="inlineStr">
+      <c r="H29" s="21" t="inlineStr">
         <is>
           <t>Dryad 공개 Excel 원자료+README. 비식별 참가자별 설문·생리 자료. 파일 존재 직접 확인</t>
         </is>
       </c>
-      <c r="H29" s="21" t="inlineStr">
+      <c r="I29" s="21" t="inlineStr">
         <is>
           <t>https://datadryad.org/dataset/doi:10.5061/dryad.mpg4f4r0v</t>
         </is>
       </c>
-      <c r="I29" s="21" t="inlineStr">
+      <c r="J29" s="21" t="inlineStr">
         <is>
           <t>https://pmc.ncbi.nlm.nih.gov/articles/PMC9873947/</t>
         </is>
       </c>
-      <c r="J29" s="21" t="inlineStr">
+      <c r="K29" s="21" t="inlineStr">
         <is>
           <t>즉시 내려받아 코드북 확인·변수별 평가 가능성 검토</t>
         </is>
       </c>
-      <c r="K29" s="21" t="inlineStr">
+      <c r="L29" s="21" t="inlineStr">
         <is>
           <t>높음</t>
         </is>
@@ -5780,40 +5914,45 @@
       </c>
       <c r="D30" s="52" t="inlineStr">
         <is>
+          <t>관찰·설문·질적 연구</t>
+        </is>
+      </c>
+      <c r="E30" s="52" t="inlineStr">
+        <is>
           <t>30개국 색채·감정 설문</t>
         </is>
       </c>
-      <c r="E30" s="57" t="inlineStr">
+      <c r="F30" s="57" t="inlineStr">
         <is>
           <t>데이터 목록 확인·접근 미확정</t>
         </is>
       </c>
-      <c r="F30" s="52" t="inlineStr">
+      <c r="G30" s="52" t="inlineStr">
         <is>
           <t>CSV·변수설명·설문 안내 파일 목록</t>
         </is>
       </c>
-      <c r="G30" s="52" t="inlineStr">
+      <c r="H30" s="52" t="inlineStr">
         <is>
           <t>SWISSUbase 데이터셋 파일 목록(Data_Wide_v1.0.csv) 확인. 계정·접근 권한 또는 라이선스 확인 전 자유 다운로드 단정 불가</t>
         </is>
       </c>
-      <c r="H30" s="52" t="inlineStr">
+      <c r="I30" s="52" t="inlineStr">
         <is>
           <t>https://www.swissubase.ch/en/catalogue/studies/13018/latest/datasets/888/1861/overview</t>
         </is>
       </c>
-      <c r="I30" s="52" t="inlineStr">
+      <c r="J30" s="52" t="inlineStr">
         <is>
           <t>https://www.swissubase.ch/en/catalogue/studies/13018/latest/datasets/888/1861/overview</t>
         </is>
       </c>
-      <c r="J30" s="52" t="inlineStr">
+      <c r="K30" s="52" t="inlineStr">
         <is>
           <t>계정 접속 후 다운로드·재사용 권한 검증</t>
         </is>
       </c>
-      <c r="K30" s="52" t="inlineStr">
+      <c r="L30" s="52" t="inlineStr">
         <is>
           <t>높음</t>
         </is>
@@ -5837,40 +5976,45 @@
       </c>
       <c r="D31" s="21" t="inlineStr">
         <is>
+          <t>이론·개념 리뷰</t>
+        </is>
+      </c>
+      <c r="E31" s="21" t="inlineStr">
+        <is>
           <t>색채 선호 이론·실험</t>
         </is>
       </c>
-      <c r="E31" s="53" t="inlineStr">
+      <c r="F31" s="53" t="inlineStr">
         <is>
           <t>참가자 RAW 미확인</t>
         </is>
       </c>
-      <c r="F31" s="21" t="inlineStr">
+      <c r="G31" s="21" t="inlineStr">
         <is>
           <t>공개 Supporting Information PDF/DOC</t>
         </is>
       </c>
-      <c r="G31" s="21" t="inlineStr">
+      <c r="H31" s="21" t="inlineStr">
         <is>
           <t>보충 PDF·DOC는 공개. 참가자 수준 원자료가 포함됐는지는 확인되지 않음</t>
         </is>
       </c>
-      <c r="H31" s="21" t="inlineStr">
+      <c r="I31" s="21" t="inlineStr">
         <is>
           <t>https://pmc.ncbi.nlm.nih.gov/articles/PMC2889342/</t>
         </is>
       </c>
-      <c r="I31" s="21" t="inlineStr">
+      <c r="J31" s="21" t="inlineStr">
         <is>
           <t>https://pmc.ncbi.nlm.nih.gov/articles/PMC2889342/</t>
         </is>
       </c>
-      <c r="J31" s="21" t="inlineStr">
+      <c r="K31" s="21" t="inlineStr">
         <is>
           <t>보충파일 열어 실제 숫자 행·변수 확인</t>
         </is>
       </c>
-      <c r="K31" s="21" t="inlineStr">
+      <c r="L31" s="21" t="inlineStr">
         <is>
           <t>높음</t>
         </is>
@@ -5894,40 +6038,45 @@
       </c>
       <c r="D32" s="52" t="inlineStr">
         <is>
+          <t>준실험·비무작위 비교</t>
+        </is>
+      </c>
+      <c r="E32" s="52" t="inlineStr">
+        <is>
           <t>색채 제시 방식 비교실험</t>
         </is>
       </c>
-      <c r="E32" s="53" t="inlineStr">
+      <c r="F32" s="53" t="inlineStr">
         <is>
           <t>참가자 RAW 미확인</t>
         </is>
       </c>
-      <c r="F32" s="52" t="inlineStr">
+      <c r="G32" s="52" t="inlineStr">
         <is>
           <t>공개 보충 PDF</t>
         </is>
       </c>
-      <c r="G32" s="52" t="inlineStr">
+      <c r="H32" s="52" t="inlineStr">
         <is>
           <t>PMC에 Supplemental PDF 존재. 참가자별 원응답 원자료 여부는 미확인</t>
         </is>
       </c>
-      <c r="H32" s="52" t="inlineStr">
+      <c r="I32" s="52" t="inlineStr">
         <is>
           <t>https://pmc.ncbi.nlm.nih.gov/articles/PMC7027086/</t>
         </is>
       </c>
-      <c r="I32" s="52" t="inlineStr">
+      <c r="J32" s="52" t="inlineStr">
         <is>
           <t>https://pmc.ncbi.nlm.nih.gov/articles/PMC7027086/</t>
         </is>
       </c>
-      <c r="J32" s="52" t="inlineStr">
+      <c r="K32" s="52" t="inlineStr">
         <is>
           <t>보충파일 확인 후 저자 데이터 요청</t>
         </is>
       </c>
-      <c r="K32" s="52" t="inlineStr">
+      <c r="L32" s="52" t="inlineStr">
         <is>
           <t>높음</t>
         </is>
@@ -5951,36 +6100,41 @@
       </c>
       <c r="D33" s="21" t="inlineStr">
         <is>
+          <t>체계적 고찰·메타분석</t>
+        </is>
+      </c>
+      <c r="E33" s="21" t="inlineStr">
+        <is>
           <t>체계적 고찰</t>
         </is>
       </c>
-      <c r="E33" s="51" t="inlineStr">
+      <c r="F33" s="51" t="inlineStr">
         <is>
           <t>리뷰/이론 (IPD 비대상)</t>
         </is>
       </c>
-      <c r="F33" s="21" t="inlineStr">
+      <c r="G33" s="21" t="inlineStr">
         <is>
           <t>문헌고찰의 출판 본문</t>
         </is>
       </c>
-      <c r="G33" s="21" t="inlineStr">
+      <c r="H33" s="21" t="inlineStr">
         <is>
           <t>옛 P04·P09 두 행이 같은 리뷰(Ohly et al., 2016)로 확인되어 한 행으로 통합(2026-10-23). IPD 연구 아님</t>
         </is>
       </c>
-      <c r="H33" s="21" t="n"/>
-      <c r="I33" s="21" t="inlineStr">
+      <c r="I33" s="21" t="n"/>
+      <c r="J33" s="21" t="inlineStr">
         <is>
           <t>https://doi.org/10.1080/10937404.2016.1196155</t>
         </is>
       </c>
-      <c r="J33" s="21" t="inlineStr">
+      <c r="K33" s="21" t="inlineStr">
         <is>
           <t>없음(중복 통합 완료)</t>
         </is>
       </c>
-      <c r="K33" s="21" t="inlineStr">
+      <c r="L33" s="21" t="inlineStr">
         <is>
           <t>높음</t>
         </is>
@@ -6004,28 +6158,33 @@
       </c>
       <c r="D34" s="52" t="inlineStr">
         <is>
+          <t>관찰·설문·질적 연구</t>
+        </is>
+      </c>
+      <c r="E34" s="52" t="inlineStr">
+        <is>
           <t>한국어 문헌</t>
         </is>
       </c>
-      <c r="E34" s="58" t="inlineStr">
+      <c r="F34" s="58" t="inlineStr">
         <is>
           <t>서지 확인 필요</t>
         </is>
       </c>
-      <c r="F34" s="52" t="n"/>
-      <c r="G34" s="52" t="inlineStr">
+      <c r="G34" s="52" t="n"/>
+      <c r="H34" s="52" t="inlineStr">
         <is>
           <t>저자·연도는 36편 근거 목록 기준으로 확인(2026-10-23). DOI·학술지 정보는 아직 확인되지 않아 RAW 조사 전</t>
         </is>
       </c>
-      <c r="H34" s="52" t="n"/>
       <c r="I34" s="52" t="n"/>
-      <c r="J34" s="52" t="inlineStr">
+      <c r="J34" s="52" t="n"/>
+      <c r="K34" s="52" t="inlineStr">
         <is>
           <t>DOI·학술지 정보 확인 후 RAW 조사</t>
         </is>
       </c>
-      <c r="K34" s="52" t="inlineStr">
+      <c r="L34" s="52" t="inlineStr">
         <is>
           <t>높음</t>
         </is>
@@ -6043,12 +6202,13 @@
       <c r="I35" s="1" t="n"/>
       <c r="J35" s="1" t="n"/>
       <c r="K35" s="1" t="n"/>
+      <c r="L35" s="1" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="A3:K3"/>
+    <mergeCell ref="A2:L2"/>
+    <mergeCell ref="A3:L3"/>
+    <mergeCell ref="A1:L1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>